<commit_message>
+  Add lock level limited when update weapon.
</commit_message>
<xml_diff>
--- a/Tool/data/Gacha.xlsx
+++ b/Tool/data/Gacha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Banners" sheetId="1" r:id="rId1"/>
@@ -600,6 +600,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -791,7 +794,7 @@
         <v>20</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D3" t="b">
         <v>0</v>
@@ -891,7 +894,7 @@
         <v>25</v>
       </c>
       <c r="C8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D8" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
+ Add more character in game
</commit_message>
<xml_diff>
--- a/Tool/data/Gacha.xlsx
+++ b/Tool/data/Gacha.xlsx
@@ -9,19 +9,19 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Banners" sheetId="1" r:id="rId1"/>
     <sheet name="Rates" sheetId="2" r:id="rId2"/>
     <sheet name="Pools" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="43">
   <si>
     <t>BannerID</t>
   </si>
@@ -90,9 +90,6 @@
   </si>
   <si>
     <t>ShaWujing</t>
-  </si>
-  <si>
-    <t>DragonKing</t>
   </si>
   <si>
     <t>ThirdPrinceNezha</t>
@@ -550,7 +547,7 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -573,7 +570,7 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
         <v>11</v>
@@ -737,7 +734,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
@@ -854,13 +851,13 @@
         <v>23</v>
       </c>
       <c r="C6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6">
         <v>100</v>
@@ -874,13 +871,13 @@
         <v>24</v>
       </c>
       <c r="C7">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D7" t="b">
         <v>0</v>
       </c>
       <c r="E7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7">
         <v>100</v>
@@ -894,13 +891,13 @@
         <v>25</v>
       </c>
       <c r="C8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D8" t="b">
         <v>0</v>
       </c>
       <c r="E8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8">
         <v>100</v>
@@ -908,7 +905,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
         <v>26</v>
@@ -917,7 +914,7 @@
         <v>5</v>
       </c>
       <c r="D9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
@@ -937,7 +934,7 @@
         <v>5</v>
       </c>
       <c r="D10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
@@ -974,13 +971,13 @@
         <v>29</v>
       </c>
       <c r="C12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12">
         <v>100</v>
@@ -994,13 +991,13 @@
         <v>30</v>
       </c>
       <c r="C13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13">
         <v>100</v>
@@ -1014,13 +1011,13 @@
         <v>31</v>
       </c>
       <c r="C14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14">
         <v>100</v>
@@ -1034,10 +1031,10 @@
         <v>32</v>
       </c>
       <c r="C15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -1054,10 +1051,10 @@
         <v>33</v>
       </c>
       <c r="C16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -1074,10 +1071,10 @@
         <v>34</v>
       </c>
       <c r="C17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -1094,7 +1091,7 @@
         <v>35</v>
       </c>
       <c r="C18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D18" t="b">
         <v>0</v>
@@ -1114,7 +1111,7 @@
         <v>36</v>
       </c>
       <c r="C19">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D19" t="b">
         <v>0</v>
@@ -1134,13 +1131,13 @@
         <v>37</v>
       </c>
       <c r="C20">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D20" t="b">
         <v>0</v>
       </c>
       <c r="E20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20">
         <v>100</v>
@@ -1154,13 +1151,13 @@
         <v>38</v>
       </c>
       <c r="C21">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F21">
         <v>100</v>
@@ -1174,13 +1171,13 @@
         <v>39</v>
       </c>
       <c r="C22">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22">
         <v>100</v>
@@ -1203,26 +1200,6 @@
         <v>1</v>
       </c>
       <c r="F23">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>10</v>
-      </c>
-      <c r="B24" t="s">
-        <v>41</v>
-      </c>
-      <c r="C24">
-        <v>5</v>
-      </c>
-      <c r="D24" t="b">
-        <v>0</v>
-      </c>
-      <c r="E24" t="b">
-        <v>1</v>
-      </c>
-      <c r="F24">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
+ Fix some bug and update big weapon icon
</commit_message>
<xml_diff>
--- a/Tool/data/Gacha.xlsx
+++ b/Tool/data/Gacha.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="45">
   <si>
     <t>BannerID</t>
   </si>
@@ -150,6 +150,12 @@
   </si>
   <si>
     <t>STR_CHARACTER_BANNER_TITLE</t>
+  </si>
+  <si>
+    <t>LiJing</t>
+  </si>
+  <si>
+    <t>ErlangShen</t>
   </si>
 </sst>
 </file>
@@ -516,7 +522,9 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -734,13 +742,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -1203,6 +1212,46 @@
         <v>100</v>
       </c>
     </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24">
+        <v>4</v>
+      </c>
+      <c r="D24" t="b">
+        <v>1</v>
+      </c>
+      <c r="E24" t="b">
+        <v>0</v>
+      </c>
+      <c r="F24">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25">
+        <v>5</v>
+      </c>
+      <c r="D25" t="b">
+        <v>1</v>
+      </c>
+      <c r="E25" t="b">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>